<commit_message>
fix: refine stage groups, template download, live media detection and rules publish script
</commit_message>
<xml_diff>
--- a/templates/活动规则标准导入模板.xlsx
+++ b/templates/活动规则标准导入模板.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="69">
   <si>
     <t>活动名称</t>
   </si>
@@ -184,22 +184,13 @@
     <t>#爱他美奇迹绿罐</t>
   </si>
   <si>
-    <t>IFFO：P段/1段</t>
-  </si>
-  <si>
     <t>IFFO</t>
   </si>
   <si>
     <t>#新生儿奶粉</t>
   </si>
   <si>
-    <t>IFFO：2段</t>
-  </si>
-  <si>
     <t>#二段奶粉推荐</t>
-  </si>
-  <si>
-    <t>GUM：3段/4段/1+段/2+段</t>
   </si>
   <si>
     <t>GUM</t>
@@ -714,7 +705,7 @@
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -751,7 +742,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>26</v>
       </c>
@@ -762,7 +753,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>28</v>
       </c>
@@ -773,7 +764,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>30</v>
       </c>
@@ -784,7 +775,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>32</v>
       </c>
@@ -795,7 +786,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>34</v>
       </c>
@@ -809,7 +800,7 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -869,7 +860,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>12</v>
       </c>
@@ -1058,7 +1049,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>12</v>
       </c>
@@ -1066,10 +1057,10 @@
         <v>56</v>
       </c>
       <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" t="s">
         <v>57</v>
-      </c>
-      <c r="E8" t="s">
-        <v>58</v>
       </c>
       <c r="F8" t="s">
         <v>47</v>
@@ -1093,18 +1084,18 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F9" t="s">
         <v>47</v>
@@ -1128,18 +1119,18 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E10" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F10" t="s">
         <v>47</v>
@@ -1166,7 +1157,7 @@
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1185,10 +1176,10 @@
         <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -1196,10 +1187,10 @@
         <v>26</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1207,10 +1198,10 @@
         <v>28</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1218,10 +1209,10 @@
         <v>30</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1229,10 +1220,10 @@
         <v>32</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1240,15 +1231,15 @@
         <v>34</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:C1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>